<commit_message>
Cập nhập thông tin thành viên
</commit_message>
<xml_diff>
--- a/information_member/informations_team.xlsx
+++ b/information_member/informations_team.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\OneDrive\Desktop\FPTPolytechnic\DATN-NghienData-develop\DATN-NghienData\information_member\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\OneDrive\Desktop\FPTPolytechnic\DATN\datag\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44A6F888-B1FA-4410-9B5D-C47C331E0138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE2ADC44-2E7C-489C-B25D-9D9D07DD8F36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2928" yWindow="2928" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INFOR" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="38">
   <si>
     <t>STT</t>
   </si>
@@ -108,6 +108,9 @@
     <t>0349570720</t>
   </si>
   <si>
+    <t xml:space="preserve"> 0969066757</t>
+  </si>
+  <si>
     <t>0354663206</t>
   </si>
   <si>
@@ -115,6 +118,27 @@
   </si>
   <si>
     <t>0356316746</t>
+  </si>
+  <si>
+    <t>MSV</t>
+  </si>
+  <si>
+    <t>PS45187</t>
+  </si>
+  <si>
+    <t>PS44508</t>
+  </si>
+  <si>
+    <t>PS45279</t>
+  </si>
+  <si>
+    <t>PS43939</t>
+  </si>
+  <si>
+    <t>PS44334</t>
+  </si>
+  <si>
+    <t>PS45024</t>
   </si>
 </sst>
 </file>
@@ -472,16 +496,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="21.33203125" customWidth="1"/>
     <col min="5" max="5" width="45.77734375" customWidth="1"/>
     <col min="6" max="6" width="17.33203125" style="6" customWidth="1"/>
+    <col min="7" max="7" width="19.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -500,8 +525,11 @@
       <c r="F1" s="4" t="s">
         <v>24</v>
       </c>
+      <c r="G1" s="3" t="s">
+        <v>31</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -518,10 +546,13 @@
         <v>14</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -540,8 +571,11 @@
       <c r="F3" s="5" t="s">
         <v>26</v>
       </c>
+      <c r="G3" s="1" t="s">
+        <v>32</v>
+      </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -558,10 +592,13 @@
         <v>16</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -578,10 +615,13 @@
         <v>15</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>25</v>
+        <v>27</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -600,8 +640,11 @@
       <c r="F6" s="5" t="s">
         <v>25</v>
       </c>
+      <c r="G6" s="1" t="s">
+        <v>37</v>
+      </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -618,7 +661,10 @@
         <v>17</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>